<commit_message>
Fill dept, project and employee codes in electricity upload file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기요금_지출결의서_업로드_26.10.xlsx
+++ b/out/전기요금_지출결의서_업로드_26.10.xlsx
@@ -64,7 +64,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -110,11 +110,6 @@
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,7 +173,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -217,8 +212,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -294,71 +287,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>경영기획실</author>
-  </authors>
-  <commentList>
-    <comment ref="M5" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M7" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M8" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M9" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M10" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M11" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M12" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M14" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M15" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M17" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-    <comment ref="M18" authorId="0" shapeId="0">
-      <text>
-        <t>조직개편 후 신규 부서코드 입력 필요</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1043,7 +971,7 @@
       </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
-          <t>4160</t>
+          <t>48000</t>
         </is>
       </c>
       <c r="N4" s="8" t="inlineStr">
@@ -1053,7 +981,7 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>2102012</t>
+          <t>2312011</t>
         </is>
       </c>
     </row>
@@ -1099,9 +1027,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M5" s="24" t="n"/>
-      <c r="N5" s="24" t="n"/>
-      <c r="O5" s="25" t="n"/>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>46300</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>2307011</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1147,7 +1087,7 @@
       </c>
       <c r="M6" s="8" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>46000</t>
         </is>
       </c>
       <c r="N6" s="8" t="inlineStr">
@@ -1203,9 +1143,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M7" s="24" t="n"/>
-      <c r="N7" s="24" t="n"/>
-      <c r="O7" s="25" t="n"/>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>46000</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>2104012</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1249,9 +1201,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="25" t="n"/>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>46000</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>2408191</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1295,9 +1259,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M9" s="24" t="n"/>
-      <c r="N9" s="24" t="n"/>
-      <c r="O9" s="25" t="n"/>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>46100</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>2608181</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1341,9 +1317,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M10" s="24" t="n"/>
-      <c r="N10" s="24" t="n"/>
-      <c r="O10" s="25" t="n"/>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>46200</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>2208016</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1387,9 +1375,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M11" s="24" t="n"/>
-      <c r="N11" s="24" t="n"/>
-      <c r="O11" s="25" t="n"/>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>46200</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>2312111</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1433,9 +1433,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M12" s="24" t="n"/>
-      <c r="N12" s="24" t="n"/>
-      <c r="O12" s="25" t="n"/>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>46200</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>2208011</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1481,7 +1493,7 @@
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="N13" s="8" t="inlineStr">
@@ -1537,9 +1549,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M14" s="24" t="n"/>
-      <c r="N14" s="24" t="n"/>
-      <c r="O14" s="25" t="n"/>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>241203</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1583,9 +1607,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M15" s="24" t="n"/>
-      <c r="N15" s="24" t="n"/>
-      <c r="O15" s="25" t="n"/>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>2606101</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1631,7 +1667,7 @@
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>3600</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
@@ -1687,9 +1723,21 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M17" s="24" t="n"/>
-      <c r="N17" s="24" t="n"/>
-      <c r="O17" s="25" t="n"/>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>45400</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>2102012</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1733,13 +1781,24 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M18" s="24" t="n"/>
-      <c r="N18" s="24" t="n"/>
-      <c r="O18" s="25" t="n"/>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>45300</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>0000000008</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>2403181</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use team-level department codes in electricity upload file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기요금_지출결의서_업로드_26.10.xlsx
+++ b/out/전기요금_지출결의서_업로드_26.10.xlsx
@@ -64,7 +64,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +110,11 @@
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -173,7 +178,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -212,6 +217,7 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -287,6 +293,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>경영기획실</author>
+  </authors>
+  <commentList>
+    <comment ref="M12" authorId="0" shapeId="0">
+      <text>
+        <t>부서코드표에 영업기획팀이 사업지원팀과 같은 46020으로 되어 있음 – 46220 등 오기 여부 확인</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1145,7 +1166,7 @@
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
-          <t>46000</t>
+          <t>46010</t>
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr">
@@ -1203,7 +1224,7 @@
       </c>
       <c r="M8" s="8" t="inlineStr">
         <is>
-          <t>46000</t>
+          <t>46020</t>
         </is>
       </c>
       <c r="N8" s="8" t="inlineStr">
@@ -1377,7 +1398,7 @@
       </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
-          <t>46200</t>
+          <t>46210</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
@@ -1433,9 +1454,9 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
-        <is>
-          <t>46200</t>
+      <c r="M12" s="24" t="inlineStr">
+        <is>
+          <t>46020</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
@@ -1551,7 +1572,7 @@
       </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>50100</t>
         </is>
       </c>
       <c r="N14" s="8" t="inlineStr">
@@ -1609,7 +1630,7 @@
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>50200</t>
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr">
@@ -1800,5 +1821,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix 영업기획팀 department code to 46220
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM2YJqCagBbEuBH1oLpGAS
</commit_message>
<xml_diff>
--- a/out/전기요금_지출결의서_업로드_26.10.xlsx
+++ b/out/전기요금_지출결의서_업로드_26.10.xlsx
@@ -64,7 +64,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -110,11 +110,6 @@
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,7 +173,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -217,7 +212,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -293,21 +287,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>경영기획실</author>
-  </authors>
-  <commentList>
-    <comment ref="M12" authorId="0" shapeId="0">
-      <text>
-        <t>부서코드표에 영업기획팀이 사업지원팀과 같은 46020으로 되어 있음 – 46220 등 오기 여부 확인</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1454,9 +1433,9 @@
           <t>20261102</t>
         </is>
       </c>
-      <c r="M12" s="24" t="inlineStr">
-        <is>
-          <t>46020</t>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>46220</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
@@ -1821,6 +1800,5 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>